<commit_message>
SOV com cores fixas por ator, abas "Produtos Globo", menções por rede na mídia espontânea
- Share of Voice: cor fixa por ator (nome normalizado sem acento/caixa),
  CNN azul, Globo laranja, Outros cinza; paleta reserva pra atores novos
- Diagnóstico e Aprendizados: rótulo "GloboNews" vira "Produtos Globo"
  (eixo na planilha continua "globonews")
- Nova aba REDES_ESPONTANEA (data, rede, mencoes) alimenta painel
  "Menções por rede" abaixo dos Big Numbers de mídia espontânea
- Helper bars() compartilhado entre os dois painéis de barras
- Template xlsx e gerador atualizados com a aba nova

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Planilha_Dash_Eleicoes_TEMPLATE.xlsx
+++ b/Planilha_Dash_Eleicoes_TEMPLATE.xlsx
@@ -12,15 +12,16 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PLATAFORMAS" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TOP_POSTS" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DIARIO" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SOV" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MENCOES_HORA" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NUVEM_TERMOS" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ASSOCIACOES" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="JORNALISTAS" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PROGRAMAS" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DIAGNOSTICO" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PONTOS" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="APRENDIZADOS" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="REDES_ESPONTANEA" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SOV" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MENCOES_HORA" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NUVEM_TERMOS" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ASSOCIACOES" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="JORNALISTAS" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PROGRAMAS" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DIAGNOSTICO" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PONTOS" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="APRENDIZADOS" sheetId="15" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -449,7 +450,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A23"/>
+  <dimension ref="A1:A24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="95" customWidth="1" min="1" max="1"/>
@@ -548,61 +549,68 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>SOV ........... Share of Voice: participacao de cada ator no volume (defina os atores)</t>
+          <t>REDES_ESPONTANEA  quebra das mencoes espontaneas por rede social (grafico abaixo dos Big Numbers)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>MENCOES_HORA .. volume de mencoes por hora; 'nota' destaca o pico</t>
+          <t>SOV ........... Share of Voice: participacao de cada ator no volume (defina os atores)</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>NUVEM_TERMOS .. termos + peso. 'escopo' = geral, jornalista:Nome ou programa:Nome</t>
+          <t>MENCOES_HORA .. volume de mencoes por hora; 'nota' destaca o pico</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>ASSOCIACOES ... associacao pauta x marca (ex: Debate + g1)</t>
+          <t>NUVEM_TERMOS .. termos + peso. 'escopo' = geral, jornalista:Nome ou programa:Nome</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>JORNALISTAS ... volume de mencoes por jornalista/apresentador + sentimento</t>
+          <t>ASSOCIACOES ... associacao pauta x marca (ex: Debate + g1)</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>PROGRAMAS ..... repercussao dos programas (GloboNews Debate, Central das Eleicoes)</t>
+          <t>JORNALISTAS ... volume de mencoes por jornalista/apresentador + sentimento</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>DIAGNOSTICO ... 'eixo' = globonews ou jornalistas; 'tipo' = funcionou ou nao_funcionou</t>
+          <t>PROGRAMAS ..... repercussao dos programas (GloboNews Debate, Central das Eleicoes)</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>PONTOS ........ 'tipo' = positivo ou atencao (crises/pontos de atencao entram como atencao)</t>
+          <t>DIAGNOSTICO ... 'eixo' = globonews (aparece como 'Produtos Globo': g1, GloboNews, TV Globo) ou jornalistas; 'tipo' = funcionou ou nao_funcionou</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
+        <is>
+          <t>PONTOS ........ 'tipo' = positivo ou atencao (crises/pontos de atencao entram como atencao)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
         <is>
           <t>APRENDIZADOS .. aprendizado do dia; 'eixo' = globonews ou jornalistas</t>
         </is>
@@ -614,6 +622,88 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>data</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>pauta</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>marca</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>mencoes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>06/08</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>Debate</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>g1</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>1800</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>06/08</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Entrevistas</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>GloboNews</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="n">
+        <v>2400</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -711,7 +801,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -793,7 +883,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -922,7 +1012,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1008,7 +1098,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1604,6 +1694,117 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:C6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>data</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>rede</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>mencoes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>06/08</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>X/Twitter</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="n">
+        <v>26000</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>06/08</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="n">
+        <v>12400</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>06/08</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="n">
+        <v>6100</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>06/08</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="n">
+        <v>2500</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>06/08</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="n">
+        <v>1200</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:C5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -1694,7 +1895,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1788,7 +1989,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1908,86 +2109,4 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:D3"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="2" t="inlineStr">
-        <is>
-          <t>data</t>
-        </is>
-      </c>
-      <c r="B1" s="2" t="inlineStr">
-        <is>
-          <t>pauta</t>
-        </is>
-      </c>
-      <c r="C1" s="2" t="inlineStr">
-        <is>
-          <t>marca</t>
-        </is>
-      </c>
-      <c r="D1" s="2" t="inlineStr">
-        <is>
-          <t>mencoes</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="3" t="inlineStr">
-        <is>
-          <t>06/08</t>
-        </is>
-      </c>
-      <c r="B2" s="3" t="inlineStr">
-        <is>
-          <t>Debate</t>
-        </is>
-      </c>
-      <c r="C2" s="3" t="inlineStr">
-        <is>
-          <t>g1</t>
-        </is>
-      </c>
-      <c r="D2" s="3" t="n">
-        <v>1800</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>06/08</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>Entrevistas</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>GloboNews</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="n">
-        <v>2400</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>